<commit_message>
Auto update 2026-09-02 09:43:51
</commit_message>
<xml_diff>
--- a/photo_links.xlsx
+++ b/photo_links.xlsx
@@ -466,14 +466,14 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405008\001_image_53405008.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405008\001_image_53405008.jpg</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F2" t="n">
-        <v>732</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="3">
@@ -494,14 +494,14 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405020\001_image_53405020.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405020\001_image_53405020.jpg</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F3" t="n">
-        <v>732</v>
+        <v>1088</v>
       </c>
     </row>
     <row r="4">
@@ -522,14 +522,14 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405064\001_image_53405064.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405064\001_image_53405064.jpg</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F4" t="n">
-        <v>732</v>
+        <v>1109</v>
       </c>
     </row>
     <row r="5">
@@ -550,14 +550,14 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405510\001_image_53405510.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405510\001_image_53405510.jpg</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F5" t="n">
-        <v>732</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="6">
@@ -578,14 +578,14 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405515\001_image_53405515.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405515\001_image_53405515.jpg</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F6" t="n">
-        <v>732</v>
+        <v>959</v>
       </c>
     </row>
     <row r="7">
@@ -606,14 +606,14 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321510\001_image_90321510.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321510\001_image_90321510.jpg</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F7" t="n">
-        <v>732</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="8">
@@ -634,14 +634,14 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321515\001_image_90321515.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321515\001_image_90321515.jpg</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F8" t="n">
-        <v>732</v>
+        <v>848</v>
       </c>
     </row>
     <row r="9">
@@ -662,14 +662,14 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321714\001_image_90321714.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321714\001_image_90321714.jpg</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F9" t="n">
-        <v>732</v>
+        <v>935</v>
       </c>
     </row>
     <row r="10">
@@ -690,14 +690,14 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405008\2_image_53405008.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405008\2_image_53405008.jpg</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F10" t="n">
-        <v>732</v>
+        <v>1359</v>
       </c>
     </row>
     <row r="11">
@@ -718,14 +718,14 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405064\2_image_53405064.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405064\2_image_53405064.jpg</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F11" t="n">
-        <v>732</v>
+        <v>1109</v>
       </c>
     </row>
     <row r="12">
@@ -746,14 +746,14 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405510\2_image_53405510.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405510\2_image_53405510.jpg</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F12" t="n">
-        <v>732</v>
+        <v>945</v>
       </c>
     </row>
     <row r="13">
@@ -774,14 +774,14 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405515\2_image_53405515.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405515\2_image_53405515.jpg</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F13" t="n">
-        <v>732</v>
+        <v>1373</v>
       </c>
     </row>
     <row r="14">
@@ -802,14 +802,14 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321510\2_image_90321510.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321510\2_image_90321510.jpg</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F14" t="n">
-        <v>732</v>
+        <v>904</v>
       </c>
     </row>
     <row r="15">
@@ -830,14 +830,14 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321515\2_image_90321515.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321515\2_image_90321515.jpg</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F15" t="n">
-        <v>732</v>
+        <v>872</v>
       </c>
     </row>
     <row r="16">
@@ -858,14 +858,14 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321714\2_image_90321714.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321714\2_image_90321714.jpg</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F16" t="n">
-        <v>732</v>
+        <v>891</v>
       </c>
     </row>
     <row r="17">
@@ -886,14 +886,14 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405008\3_image_53405008.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405008\3_image_53405008.jpg</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F17" t="n">
-        <v>732</v>
+        <v>1106</v>
       </c>
     </row>
     <row r="18">
@@ -914,14 +914,14 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405020\3_image_53405020.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405020\3_image_53405020.jpg</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F18" t="n">
-        <v>732</v>
+        <v>989</v>
       </c>
     </row>
     <row r="19">
@@ -942,14 +942,14 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405064\3_image_53405064.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405064\3_image_53405064.jpg</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F19" t="n">
-        <v>732</v>
+        <v>760</v>
       </c>
     </row>
     <row r="20">
@@ -970,14 +970,14 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405515\3_image_53405515.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405515\3_image_53405515.jpg</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F20" t="n">
-        <v>732</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="21">
@@ -998,14 +998,14 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321515\3_image_90321515.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321515\3_image_90321515.jpg</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F21" t="n">
-        <v>732</v>
+        <v>848</v>
       </c>
     </row>
     <row r="22">
@@ -1026,14 +1026,14 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405020\4_image_53405020.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405020\4_image_53405020.jpg</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F22" t="n">
-        <v>732</v>
+        <v>1210</v>
       </c>
     </row>
     <row r="23">
@@ -1054,14 +1054,14 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405064\4_image_53405064.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405064\4_image_53405064.jpg</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F23" t="n">
-        <v>732</v>
+        <v>904</v>
       </c>
     </row>
     <row r="24">
@@ -1082,14 +1082,14 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405510\4_image_53405510.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405510\4_image_53405510.jpg</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F24" t="n">
-        <v>732</v>
+        <v>1401</v>
       </c>
     </row>
     <row r="25">
@@ -1110,14 +1110,14 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405515\4_image_53405515.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405515\4_image_53405515.jpg</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F25" t="n">
-        <v>732</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="26">
@@ -1138,14 +1138,14 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321510\4_image_90321510.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321510\4_image_90321510.jpg</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F26" t="n">
-        <v>732</v>
+        <v>1049</v>
       </c>
     </row>
     <row r="27">
@@ -1166,14 +1166,14 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321515\4_image_90321515.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321515\4_image_90321515.jpg</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F27" t="n">
-        <v>732</v>
+        <v>898</v>
       </c>
     </row>
     <row r="28">
@@ -1194,14 +1194,14 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321714\4_image_90321714.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321714\4_image_90321714.jpg</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F28" t="n">
-        <v>732</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="29">
@@ -1222,14 +1222,14 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405008\5_image_53405008.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405008\5_image_53405008.jpg</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F29" t="n">
-        <v>732</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="30">
@@ -1250,14 +1250,14 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405020\5_image_53405020.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405020\5_image_53405020.jpg</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F30" t="n">
-        <v>732</v>
+        <v>932</v>
       </c>
     </row>
     <row r="31">
@@ -1278,14 +1278,14 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405064\5_image_53405064.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405064\5_image_53405064.jpg</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F31" t="n">
-        <v>732</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="32">
@@ -1306,14 +1306,14 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405510\5_image_53405510.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405510\5_image_53405510.jpg</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F32" t="n">
-        <v>732</v>
+        <v>1374</v>
       </c>
     </row>
     <row r="33">
@@ -1334,14 +1334,14 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405515\5_image_53405515.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405515\5_image_53405515.jpg</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F33" t="n">
-        <v>732</v>
+        <v>771</v>
       </c>
     </row>
     <row r="34">
@@ -1362,14 +1362,14 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321510\5_image_90321510.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321510\5_image_90321510.jpg</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F34" t="n">
-        <v>732</v>
+        <v>816</v>
       </c>
     </row>
     <row r="35">
@@ -1390,14 +1390,14 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321515\5_image_90321515.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321515\5_image_90321515.jpg</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F35" t="n">
-        <v>732</v>
+        <v>1431</v>
       </c>
     </row>
     <row r="36">
@@ -1418,14 +1418,14 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321714\5_image_90321714.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321714\5_image_90321714.jpg</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F36" t="n">
-        <v>732</v>
+        <v>1515</v>
       </c>
     </row>
     <row r="37">
@@ -1446,14 +1446,14 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405008\6_image_53405008.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405008\6_image_53405008.jpg</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F37" t="n">
-        <v>732</v>
+        <v>1502</v>
       </c>
     </row>
     <row r="38">
@@ -1474,14 +1474,14 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405020\6_image_53405020.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405020\6_image_53405020.jpg</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F38" t="n">
-        <v>732</v>
+        <v>1404</v>
       </c>
     </row>
     <row r="39">
@@ -1502,14 +1502,14 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405064\6_image_53405064.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405064\6_image_53405064.jpg</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F39" t="n">
-        <v>732</v>
+        <v>1271</v>
       </c>
     </row>
     <row r="40">
@@ -1530,14 +1530,14 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405510\6_image_53405510.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405510\6_image_53405510.jpg</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F40" t="n">
-        <v>732</v>
+        <v>1455</v>
       </c>
     </row>
     <row r="41">
@@ -1558,14 +1558,14 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405515\6_image_53405515.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405515\6_image_53405515.jpg</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F41" t="n">
-        <v>732</v>
+        <v>972</v>
       </c>
     </row>
     <row r="42">
@@ -1586,14 +1586,14 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321510\6_image_90321510.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321510\6_image_90321510.jpg</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F42" t="n">
-        <v>732</v>
+        <v>746</v>
       </c>
     </row>
     <row r="43">
@@ -1614,14 +1614,14 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321515\6_image_90321515.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321515\6_image_90321515.jpg</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F43" t="n">
-        <v>732</v>
+        <v>868</v>
       </c>
     </row>
     <row r="44">
@@ -1642,14 +1642,14 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321714\6_image_90321714.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321714\6_image_90321714.jpg</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F44" t="n">
-        <v>732</v>
+        <v>854</v>
       </c>
     </row>
     <row r="45">
@@ -1670,14 +1670,14 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405008\7_image_53405008.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405008\7_image_53405008.jpg</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F45" t="n">
-        <v>732</v>
+        <v>1561</v>
       </c>
     </row>
     <row r="46">
@@ -1698,14 +1698,14 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405020\7_image_53405020.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405020\7_image_53405020.jpg</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F46" t="n">
-        <v>732</v>
+        <v>921</v>
       </c>
     </row>
     <row r="47">
@@ -1726,14 +1726,14 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405064\7_image_53405064.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405064\7_image_53405064.jpg</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F47" t="n">
-        <v>732</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="48">
@@ -1754,14 +1754,14 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405510\7_image_53405510.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405510\7_image_53405510.jpg</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F48" t="n">
-        <v>732</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="49">
@@ -1782,14 +1782,14 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321510\7_image_90321510.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321510\7_image_90321510.jpg</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F49" t="n">
-        <v>732</v>
+        <v>746</v>
       </c>
     </row>
     <row r="50">
@@ -1810,14 +1810,14 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321515\7_image_90321515.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321515\7_image_90321515.jpg</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F50" t="n">
-        <v>732</v>
+        <v>724</v>
       </c>
     </row>
     <row r="51">
@@ -1838,14 +1838,14 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321714\7_image_90321714.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321714\7_image_90321714.jpg</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F51" t="n">
-        <v>732</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="52">
@@ -1866,14 +1866,14 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405008\8_image_53405008.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405008\8_image_53405008.jpg</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F52" t="n">
-        <v>732</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="53">
@@ -1894,14 +1894,14 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405020\8_image_53405020.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405020\8_image_53405020.jpg</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F53" t="n">
-        <v>732</v>
+        <v>1673</v>
       </c>
     </row>
     <row r="54">
@@ -1922,14 +1922,14 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405064\8_image_53405064.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405064\8_image_53405064.jpg</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F54" t="n">
-        <v>732</v>
+        <v>926</v>
       </c>
     </row>
     <row r="55">
@@ -1950,14 +1950,14 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405510\8_image_53405510.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405510\8_image_53405510.jpg</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F55" t="n">
-        <v>732</v>
+        <v>999</v>
       </c>
     </row>
     <row r="56">
@@ -1978,14 +1978,14 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405515\8_image_53405515.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405515\8_image_53405515.jpg</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F56" t="n">
-        <v>732</v>
+        <v>1431</v>
       </c>
     </row>
     <row r="57">
@@ -2006,14 +2006,14 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321510\008_image_90321510.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321510\008_image_90321510.jpg</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F57" t="n">
-        <v>732</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="58">
@@ -2034,14 +2034,14 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321515\8_image_90321515.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321515\8_image_90321515.jpg</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F58" t="n">
-        <v>732</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="59">
@@ -2062,14 +2062,14 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321714\8_image_90321714.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321714\8_image_90321714.jpg</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F59" t="n">
-        <v>732</v>
+        <v>746</v>
       </c>
     </row>
     <row r="60">
@@ -2090,14 +2090,14 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405008\9_image_53405008.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405008\9_image_53405008.jpg</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F60" t="n">
-        <v>732</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="61">
@@ -2118,14 +2118,14 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405020\9_image_53405020.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405020\9_image_53405020.jpg</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F61" t="n">
-        <v>732</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="62">
@@ -2146,14 +2146,14 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405064\9_image_53405064.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405064\9_image_53405064.jpg</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F62" t="n">
-        <v>732</v>
+        <v>921</v>
       </c>
     </row>
     <row r="63">
@@ -2174,14 +2174,14 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405510\9_image_53405510.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405510\9_image_53405510.jpg</t>
         </is>
       </c>
       <c r="E63" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F63" t="n">
-        <v>732</v>
+        <v>811</v>
       </c>
     </row>
     <row r="64">
@@ -2202,14 +2202,14 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405515\9_image_53405515.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405515\9_image_53405515.jpg</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F64" t="n">
-        <v>732</v>
+        <v>1412</v>
       </c>
     </row>
     <row r="65">
@@ -2230,14 +2230,14 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321714\9_image_90321714.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321714\9_image_90321714.jpg</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F65" t="n">
-        <v>732</v>
+        <v>746</v>
       </c>
     </row>
     <row r="66">
@@ -2258,14 +2258,14 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405008\10_image_53405008.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405008\10_image_53405008.jpg</t>
         </is>
       </c>
       <c r="E66" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F66" t="n">
-        <v>732</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="67">
@@ -2286,14 +2286,14 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405020\10_image_53405020.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405020\10_image_53405020.jpg</t>
         </is>
       </c>
       <c r="E67" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F67" t="n">
-        <v>732</v>
+        <v>900</v>
       </c>
     </row>
     <row r="68">
@@ -2314,14 +2314,14 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405510\10_image_53405510.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405510\10_image_53405510.jpg</t>
         </is>
       </c>
       <c r="E68" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F68" t="n">
-        <v>732</v>
+        <v>760</v>
       </c>
     </row>
     <row r="69">
@@ -2342,14 +2342,14 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405515\10_image_53405515.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405515\10_image_53405515.jpg</t>
         </is>
       </c>
       <c r="E69" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F69" t="n">
-        <v>732</v>
+        <v>885</v>
       </c>
     </row>
     <row r="70">
@@ -2370,14 +2370,14 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321515\10_image_90321515.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321515\10_image_90321515.jpg</t>
         </is>
       </c>
       <c r="E70" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F70" t="n">
-        <v>732</v>
+        <v>746</v>
       </c>
     </row>
     <row r="71">
@@ -2398,14 +2398,14 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321714\010_image_90321714.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321714\010_image_90321714.jpg</t>
         </is>
       </c>
       <c r="E71" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F71" t="n">
-        <v>732</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="72">
@@ -2426,14 +2426,14 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405008\11_image_53405008.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405008\11_image_53405008.jpg</t>
         </is>
       </c>
       <c r="E72" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F72" t="n">
-        <v>732</v>
+        <v>917</v>
       </c>
     </row>
     <row r="73">
@@ -2454,14 +2454,14 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405020\11_image_53405020.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405020\11_image_53405020.jpg</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F73" t="n">
-        <v>732</v>
+        <v>746</v>
       </c>
     </row>
     <row r="74">
@@ -2482,14 +2482,14 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405064\11_image_53405064.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405064\11_image_53405064.jpg</t>
         </is>
       </c>
       <c r="E74" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F74" t="n">
-        <v>732</v>
+        <v>989</v>
       </c>
     </row>
     <row r="75">
@@ -2510,14 +2510,14 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405510\11_image_53405510.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405510\11_image_53405510.jpg</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F75" t="n">
-        <v>732</v>
+        <v>746</v>
       </c>
     </row>
     <row r="76">
@@ -2538,14 +2538,14 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405515\11_image_53405515.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405515\11_image_53405515.jpg</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F76" t="n">
-        <v>732</v>
+        <v>746</v>
       </c>
     </row>
     <row r="77">
@@ -2566,14 +2566,14 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321515\11_image_90321515.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321515\11_image_90321515.jpg</t>
         </is>
       </c>
       <c r="E77" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F77" t="n">
-        <v>732</v>
+        <v>746</v>
       </c>
     </row>
     <row r="78">
@@ -2594,14 +2594,14 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405008\12_image_53405008.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405008\12_image_53405008.jpg</t>
         </is>
       </c>
       <c r="E78" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F78" t="n">
-        <v>732</v>
+        <v>746</v>
       </c>
     </row>
     <row r="79">
@@ -2622,14 +2622,14 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405020\12_image_53405020.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405020\12_image_53405020.jpg</t>
         </is>
       </c>
       <c r="E79" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F79" t="n">
-        <v>732</v>
+        <v>746</v>
       </c>
     </row>
     <row r="80">
@@ -2650,14 +2650,14 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405064\12_image_53405064.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405064\12_image_53405064.jpg</t>
         </is>
       </c>
       <c r="E80" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F80" t="n">
-        <v>732</v>
+        <v>746</v>
       </c>
     </row>
     <row r="81">
@@ -2678,14 +2678,14 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405510\12_image_53405510.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405510\12_image_53405510.jpg</t>
         </is>
       </c>
       <c r="E81" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F81" t="n">
-        <v>732</v>
+        <v>746</v>
       </c>
     </row>
     <row r="82">
@@ -2706,14 +2706,14 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405515\12_image_53405515.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405515\12_image_53405515.jpg</t>
         </is>
       </c>
       <c r="E82" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F82" t="n">
-        <v>732</v>
+        <v>746</v>
       </c>
     </row>
     <row r="83">
@@ -2734,14 +2734,14 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321515\12_image_90321515.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321515\12_image_90321515.jpg</t>
         </is>
       </c>
       <c r="E83" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F83" t="n">
-        <v>732</v>
+        <v>711</v>
       </c>
     </row>
     <row r="84">
@@ -2762,14 +2762,14 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405008\13_image_53405008.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405008\13_image_53405008.jpg</t>
         </is>
       </c>
       <c r="E84" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F84" t="n">
-        <v>732</v>
+        <v>746</v>
       </c>
     </row>
     <row r="85">
@@ -2790,14 +2790,14 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405020\13_image_53405020.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405020\13_image_53405020.jpg</t>
         </is>
       </c>
       <c r="E85" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F85" t="n">
-        <v>732</v>
+        <v>746</v>
       </c>
     </row>
     <row r="86">
@@ -2818,14 +2818,14 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405064\13_image_53405064.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405064\13_image_53405064.jpg</t>
         </is>
       </c>
       <c r="E86" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F86" t="n">
-        <v>732</v>
+        <v>746</v>
       </c>
     </row>
     <row r="87">
@@ -2846,14 +2846,14 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405510\13_image_53405510.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405510\13_image_53405510.jpg</t>
         </is>
       </c>
       <c r="E87" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F87" t="n">
-        <v>732</v>
+        <v>746</v>
       </c>
     </row>
     <row r="88">
@@ -2874,14 +2874,14 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405515\13_image_53405515.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405515\13_image_53405515.jpg</t>
         </is>
       </c>
       <c r="E88" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F88" t="n">
-        <v>732</v>
+        <v>746</v>
       </c>
     </row>
     <row r="89">
@@ -2902,14 +2902,14 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321515\13_image_90321515.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321515\13_image_90321515.jpg</t>
         </is>
       </c>
       <c r="E89" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F89" t="n">
-        <v>732</v>
+        <v>918</v>
       </c>
     </row>
     <row r="90">
@@ -2930,14 +2930,14 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405008\14_image_53405008.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405008\14_image_53405008.jpg</t>
         </is>
       </c>
       <c r="E90" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F90" t="n">
-        <v>732</v>
+        <v>746</v>
       </c>
     </row>
     <row r="91">
@@ -2958,14 +2958,14 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405020\14_image_53405020.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405020\14_image_53405020.jpg</t>
         </is>
       </c>
       <c r="E91" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F91" t="n">
-        <v>732</v>
+        <v>746</v>
       </c>
     </row>
     <row r="92">
@@ -2986,14 +2986,14 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405064\14_image_53405064.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405064\14_image_53405064.jpg</t>
         </is>
       </c>
       <c r="E92" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F92" t="n">
-        <v>732</v>
+        <v>746</v>
       </c>
     </row>
     <row r="93">
@@ -3014,14 +3014,14 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405510\014_image_53405510.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405510\014_image_53405510.jpg</t>
         </is>
       </c>
       <c r="E93" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F93" t="n">
-        <v>732</v>
+        <v>1115</v>
       </c>
     </row>
     <row r="94">
@@ -3042,14 +3042,14 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405515\14_image_53405515.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405515\14_image_53405515.jpg</t>
         </is>
       </c>
       <c r="E94" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F94" t="n">
-        <v>732</v>
+        <v>746</v>
       </c>
     </row>
     <row r="95">
@@ -3070,14 +3070,14 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\90321515\014_image_90321515.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\90321515\014_image_90321515.jpg</t>
         </is>
       </c>
       <c r="E95" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F95" t="n">
-        <v>732</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="96">
@@ -3098,14 +3098,14 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405008\015_image_53405008.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405008\015_image_53405008.jpg</t>
         </is>
       </c>
       <c r="E96" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F96" t="n">
-        <v>732</v>
+        <v>1107</v>
       </c>
     </row>
     <row r="97">
@@ -3126,14 +3126,14 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405020\15_image_53405020.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405020\15_image_53405020.jpg</t>
         </is>
       </c>
       <c r="E97" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F97" t="n">
-        <v>732</v>
+        <v>746</v>
       </c>
     </row>
     <row r="98">
@@ -3154,14 +3154,14 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405064\015_image_53405064.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405064\015_image_53405064.jpg</t>
         </is>
       </c>
       <c r="E98" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F98" t="n">
-        <v>732</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="99">
@@ -3182,14 +3182,14 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405515\015_image_53405515.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405515\015_image_53405515.jpg</t>
         </is>
       </c>
       <c r="E99" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F99" t="n">
-        <v>732</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="100">
@@ -3210,14 +3210,14 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/3 самбег посортовані\53405020\016_image_53405020.jpg</t>
+          <t>C:/Users/Asus/Desktop/1 редагування2026/385 сумки/фото/4 обрізані\53405020\016_image_53405020.jpg</t>
         </is>
       </c>
       <c r="E100" t="n">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F100" t="n">
-        <v>732</v>
+        <v>1022</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update 2026-10-30 20:56:54
</commit_message>
<xml_diff>
--- a/photo_links.xlsx
+++ b/photo_links.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F77"/>
+  <dimension ref="A1:F157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,7 +451,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BN-GC-19-g-kr</t>
+          <t>BN-IDC-1-g</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -461,25 +461,25 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-19-g-kr/001.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-1-g/001.jpg</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-19-g-kr\001_image_BN-GC-19-g-kr.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-1-g\001_image_BN-IDC-1-g.png</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1482</v>
+        <v>550</v>
       </c>
       <c r="F2" t="n">
-        <v>1061</v>
+        <v>1424</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BN-GC-19-iz</t>
+          <t>BN-IDC-2-1-beige-kr</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -489,25 +489,25 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-19-iz/001.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-1-beige-kr/001.jpg</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-19-iz\001_image_BN-GC-19-iz.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-1-beige-kr\001_image_BN-IDC-2-1-beige-kr.png</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>1482</v>
+        <v>1057</v>
       </c>
       <c r="F3" t="n">
-        <v>1062</v>
+        <v>800</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BN-GC-19-k-kr</t>
+          <t>BN-IDC-2-1-g-kr</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -517,25 +517,25 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-19-k-kr/001.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-1-g-kr/001.jpg</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-19-k-kr\001_image_BN-GC-19-k-kr.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-1-g-kr\001_image_BN-IDC-2-1-g-kr.png</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>1482</v>
+        <v>1113</v>
       </c>
       <c r="F4" t="n">
-        <v>1061</v>
+        <v>769</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BN-GC-19-o</t>
+          <t>BN-IDC-2-1-k-kr</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -545,25 +545,25 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-19-o/001.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-1-k-kr/001.jpg</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-19-o\001_image_BN-GC-19-o.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-1-k-kr\001_image_BN-IDC-2-1-k-kr.png</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>1483</v>
+        <v>1103</v>
       </c>
       <c r="F5" t="n">
-        <v>1061</v>
+        <v>809</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BN-GC-19-vin-kr</t>
+          <t>BN-IDC-2-1-malachite</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -573,25 +573,25 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-19-vin-kr/001.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-1-malachite/001.jpg</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-19-vin-kr\001_image_BN-GC-19-vin-kr.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-1-malachite\001_image_BN-IDC-2-1-malachite.png</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>1482</v>
+        <v>1144</v>
       </c>
       <c r="F6" t="n">
-        <v>1062</v>
+        <v>773</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BN-GC-28-choko</t>
+          <t>BN-IDC-2-1-navy-blue</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -601,25 +601,25 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-28-choko/001.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-1-navy-blue/001.jpg</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-28-choko\001_image_BN-GC-28-choko.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-1-navy-blue\001_image_BN-IDC-2-1-navy-blue.png</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>1498</v>
+        <v>1081</v>
       </c>
       <c r="F7" t="n">
-        <v>1050</v>
+        <v>757</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BN-GC-28-g</t>
+          <t>BN-IDC-2-1-nn</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -629,25 +629,25 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-28-g/001.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-1-nn/001.jpg</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-28-g\001_image_BN-GC-28-g.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-1-nn\001_image_BN-IDC-2-1-nn.png</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>1482</v>
+        <v>1122</v>
       </c>
       <c r="F8" t="n">
-        <v>1061</v>
+        <v>783</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BN-GC-28-k</t>
+          <t>BN-IDC-2-1-o</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -657,25 +657,25 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-28-k/001.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-1-o/001.jpg</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-28-k\001_image_BN-GC-28-k.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-1-o\001_image_BN-IDC-2-1-o.png</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>1482</v>
+        <v>1135</v>
       </c>
       <c r="F9" t="n">
-        <v>1061</v>
+        <v>775</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BN-GC-28-malachite</t>
+          <t>BN-IDC-2-1-red</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -685,25 +685,25 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-28-malachite/001.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-1-red/001.jpg</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-28-malachite\001_image_BN-GC-28-malachite.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-1-red\001_image_BN-IDC-2-1-red.png</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>1483</v>
+        <v>1040</v>
       </c>
       <c r="F10" t="n">
-        <v>1061</v>
+        <v>739</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BN-GC-7-g-kr</t>
+          <t>BN-IDC-2-2-beige-kr</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -713,25 +713,25 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-g-kr/001.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-2-beige-kr/001.jpg</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-g-kr\001_image_BN-GC-7-g-kr.jpg</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-2-beige-kr\001_image_BN-IDC-2-2-beige-kr.png</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>723</v>
+        <v>991</v>
       </c>
       <c r="F11" t="n">
-        <v>530</v>
+        <v>743</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BN-GC-7-iz</t>
+          <t>BN-IDC-2-2-choko</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -741,25 +741,25 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-iz/001.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-2-choko/001.jpg</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-iz\001_image_BN-GC-7-iz.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-2-choko\001_image_BN-IDC-2-2-choko.png</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>1482</v>
+        <v>971</v>
       </c>
       <c r="F12" t="n">
-        <v>1062</v>
+        <v>700</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BN-GC-7-k</t>
+          <t>BN-IDC-2-2-g-kr</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -769,25 +769,25 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-k/001.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-2-g-kr/001.jpg</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-k\001_image_BN-GC-7-k.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-2-g-kr\001_image_BN-IDC-2-2-g-kr.png</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>1482</v>
+        <v>1019</v>
       </c>
       <c r="F13" t="n">
-        <v>1061</v>
+        <v>730</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BN-GC-7-k-kr</t>
+          <t>BN-IDC-2-2-iz</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -797,25 +797,25 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-k-kr/001.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-2-iz/001.jpg</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-k-kr\001_image_BN-GC-7-k-kr.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-2-iz\001_image_BN-IDC-2-2-iz.png</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>1482</v>
+        <v>1015</v>
       </c>
       <c r="F14" t="n">
-        <v>1061</v>
+        <v>727</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>BN-GC-7-malachite</t>
+          <t>BN-IDC-2-2-k-kr</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -825,25 +825,25 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-malachite/001.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-2-k-kr/001.jpg</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-malachite\001_image_BN-GC-7-malachite.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-2-k-kr\001_image_BN-IDC-2-2-k-kr.png</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>1483</v>
+        <v>1059</v>
       </c>
       <c r="F15" t="n">
-        <v>1061</v>
+        <v>755</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BN-GC-7-navy-blue</t>
+          <t>BN-IDC-2-2-malachite</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -853,25 +853,25 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-navy-blue/001.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-2-malachite/001.jpg</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-navy-blue\001_image_BN-GC-7-navy-blue.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-2-malachite\001_image_BN-IDC-2-2-malachite.png</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>1482</v>
+        <v>991</v>
       </c>
       <c r="F16" t="n">
-        <v>1061</v>
+        <v>716</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>BN-GC-7-nn</t>
+          <t>BN-IDC-2-2-nn</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -881,25 +881,25 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-nn/001.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-2-nn/001.jpg</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-nn\001_image_BN-GC-7-nn.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-2-nn\001_image_BN-IDC-2-2-nn.png</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>1483</v>
+        <v>1048</v>
       </c>
       <c r="F17" t="n">
-        <v>1061</v>
+        <v>760</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>BN-GC-7-o</t>
+          <t>BN-IDC-2-2-o</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -909,25 +909,25 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-o/001.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-2-o/001.jpg</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-o\001_image_BN-GC-7-o.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-2-o\001_image_BN-IDC-2-2-o.png</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>1483</v>
+        <v>1029</v>
       </c>
       <c r="F18" t="n">
-        <v>1061</v>
+        <v>756</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>BN-GC-7-red</t>
+          <t>BN-OP-23-1-k</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -937,25 +937,25 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-red/001.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-1-k/001.jpg</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-red\001_image_BN-GC-7-red.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-1-k\001_image_BN-OP-23-1-k.png</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>1482</v>
+        <v>1149</v>
       </c>
       <c r="F19" t="n">
-        <v>1061</v>
+        <v>784</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>BN-GC-7-tiffany</t>
+          <t>BN-OP-23-1-malachite</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -965,25 +965,25 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-tiffany/001.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-1-malachite/001.jpg</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-tiffany\001_image_BN-GC-7-tiffany.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-1-malachite\001_image_BN-OP-23-1-malachite.png</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>1482</v>
+        <v>1112</v>
       </c>
       <c r="F20" t="n">
-        <v>1061</v>
+        <v>755</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>BN-GC-7-vin</t>
+          <t>BN-OP-23-1-navy-blue</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -993,25 +993,25 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-vin/001.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-1-navy-blue/001.jpg</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-vin\001_image_BN-GC-7-vin.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-1-navy-blue\001_image_BN-OP-23-1-navy-blue.png</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>1483</v>
+        <v>1023</v>
       </c>
       <c r="F21" t="n">
-        <v>1061</v>
+        <v>690</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BN-GC-7-vin-kr</t>
+          <t>BN-OP-23-beige</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1021,25 +1021,25 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-vin-kr/001.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-beige/001.jpg</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-vin-kr\001_image_BN-GC-7-vin-kr.jpg</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-beige\001_image_BN-OP-23-beige.png</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>2384</v>
+        <v>876</v>
       </c>
       <c r="F22" t="n">
-        <v>1760</v>
+        <v>588</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>BN-GC-8-g-kr</t>
+          <t>BN-OP-23-choko</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1049,25 +1049,25 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-8-g-kr/001.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-choko/001.jpg</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-8-g-kr\001_image_BN-GC-8-g-kr.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-choko\001_image_BN-OP-23-choko.png</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>1482</v>
+        <v>987</v>
       </c>
       <c r="F23" t="n">
-        <v>1061</v>
+        <v>652</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>BN-GC-8-k-kr</t>
+          <t>BN-OP-23-g</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1077,25 +1077,25 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-8-k-kr/001.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-g/001.jpg</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-8-k-kr\001_image_BN-GC-8-k-kr.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-g\001_image_BN-OP-23-g.png</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>1482</v>
+        <v>1045</v>
       </c>
       <c r="F24" t="n">
-        <v>1061</v>
+        <v>672</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>BN-GC-8-o</t>
+          <t>BN-OP-23-k</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1105,389 +1105,389 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-8-o/001.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-k/001.jpg</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-8-o\001_image_BN-GC-8-o.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-k\001_image_BN-OP-23-k.png</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>1482</v>
+        <v>874</v>
       </c>
       <c r="F25" t="n">
-        <v>1061</v>
+        <v>1111</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>BN-GC-19-g-kr</t>
+          <t>BN-OP-23-malachite</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>002.jpg</t>
+          <t>001.jpg</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-19-g-kr/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-malachite/001.jpg</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-19-g-kr\002_image_BN-GC-19-g-kr.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-malachite\001_image_BN-OP-23-malachite.png</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>1482</v>
+        <v>1070</v>
       </c>
       <c r="F26" t="n">
-        <v>1061</v>
+        <v>718</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>BN-GC-19-iz</t>
+          <t>BN-OP-23-navy-blue</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>002.jpg</t>
+          <t>001.jpg</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-19-iz/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-navy-blue/001.jpg</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-19-iz\002_image_BN-GC-19-iz.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-navy-blue\001_image_BN-OP-23-navy-blue.png</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>1483</v>
+        <v>1095</v>
       </c>
       <c r="F27" t="n">
-        <v>1061</v>
+        <v>725</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>BN-GC-19-k-kr</t>
+          <t>BN-OP-25-1-choko</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>002.jpg</t>
+          <t>001.jpg</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-19-k-kr/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-choko/001.jpg</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-19-k-kr\002_image_BN-GC-19-k-kr.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-choko\001_image_BN-OP-25-1-choko.png</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1482</v>
+        <v>854</v>
       </c>
       <c r="F28" t="n">
-        <v>1061</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>BN-GC-19-o</t>
+          <t>BN-OP-25-1-g</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>002.jpg</t>
+          <t>001.jpg</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-19-o/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-g/001.jpg</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-19-o\002_image_BN-GC-19-o.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-g\001_image_BN-OP-25-1-g.png</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>1482</v>
+        <v>844</v>
       </c>
       <c r="F29" t="n">
-        <v>1061</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>BN-GC-19-vin-kr</t>
+          <t>BN-OP-25-1-k</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>002.jpg</t>
+          <t>001.jpg</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-19-vin-kr/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-k/001.jpg</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-19-vin-kr\002_image_BN-GC-19-vin-kr.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-k\001_image_BN-OP-25-1-k.png</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>1483</v>
+        <v>828</v>
       </c>
       <c r="F30" t="n">
-        <v>1061</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>BN-GC-28-choko</t>
+          <t>BN-OP-25-1-light-beige</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>002.jpg</t>
+          <t>001.jpg</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-28-choko/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-light-beige/001.jpg</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-28-choko\002_image_BN-GC-28-choko.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-light-beige\001_image_BN-OP-25-1-light-beige.png</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>1483</v>
+        <v>826</v>
       </c>
       <c r="F31" t="n">
-        <v>1061</v>
+        <v>983</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>BN-GC-28-g</t>
+          <t>BN-OP-25-1-malachite</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>002.jpg</t>
+          <t>001.jpg</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-28-g/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-malachite/001.jpg</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-28-g\002_image_BN-GC-28-g.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-malachite\001_image_BN-OP-25-1-malachite.png</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>1462</v>
+        <v>808</v>
       </c>
       <c r="F32" t="n">
-        <v>1076</v>
+        <v>930</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>BN-GC-28-k</t>
+          <t>BN-OP-25-1-navy-blue</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>002.jpg</t>
+          <t>001.jpg</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-28-k/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-navy-blue/001.jpg</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-28-k\002_image_BN-GC-28-k.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-navy-blue\001_image_BN-OP-25-1-navy-blue.jpg</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>1460</v>
+        <v>530</v>
       </c>
       <c r="F33" t="n">
-        <v>1077</v>
+        <v>633</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>BN-GC-28-malachite</t>
+          <t>BN-OP-25-g-kr</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>002.jpg</t>
+          <t>001.jpg</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-28-malachite/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-g-kr/001.jpg</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-28-malachite\002_image_BN-GC-28-malachite.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-g-kr\001_image_BN-OP-25-g-kr.png</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>1482</v>
+        <v>782</v>
       </c>
       <c r="F34" t="n">
-        <v>1061</v>
+        <v>958</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>BN-GC-7-g-kr</t>
+          <t>BN-OP-25-malachite</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>002.jpg</t>
+          <t>001.jpg</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-g-kr/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-malachite/001.jpg</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-g-kr\002_image_BN-GC-7-g-kr.jpg</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-malachite\001_image_BN-OP-25-malachite.png</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>726</v>
+        <v>798</v>
       </c>
       <c r="F35" t="n">
-        <v>530</v>
+        <v>958</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>BN-GC-7-iz</t>
+          <t>BN-OP-25-navy-blue</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>002.jpg</t>
+          <t>001.jpg</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-iz/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-navy-blue/001.jpg</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-iz\002_image_BN-GC-7-iz.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-navy-blue\001_image_BN-OP-25-navy-blue.png</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>1482</v>
+        <v>787</v>
       </c>
       <c r="F36" t="n">
-        <v>1061</v>
+        <v>941</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>BN-GC-7-k</t>
+          <t>BN-OP-26-k</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>002.jpg</t>
+          <t>001.jpg</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-k/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-26-k/001.jpg</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-k\002_image_BN-GC-7-k.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-26-k\001_image_BN-OP-26-k.png</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>1482</v>
+        <v>926</v>
       </c>
       <c r="F37" t="n">
-        <v>1062</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>BN-GC-7-k-kr</t>
+          <t>BN-OP-26-light</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>002.jpg</t>
+          <t>001.jpg</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-k-kr/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-26-light/001.jpg</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-k-kr\002_image_BN-GC-7-k-kr.jpg</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-26-light\001_image_BN-OP-26-light.png</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>2752</v>
+        <v>944</v>
       </c>
       <c r="F38" t="n">
-        <v>1536</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>BN-GC-7-malachite</t>
+          <t>BN-IDC-1-g</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1497,25 +1497,25 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-malachite/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-1-g/002.jpg</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-malachite\002_image_BN-GC-7-malachite.jpg</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-1-g\2_image_BN-IDC-1-g.png</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>2752</v>
+        <v>530</v>
       </c>
       <c r="F39" t="n">
-        <v>1536</v>
+        <v>1720</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>BN-GC-7-navy-blue</t>
+          <t>BN-IDC-2-1-beige-kr</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1525,25 +1525,25 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-navy-blue/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-1-beige-kr/002.jpg</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-navy-blue\002_image_BN-GC-7-navy-blue.jpg</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-1-beige-kr\2_image_BN-IDC-2-1-beige-kr.png</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>2752</v>
+        <v>1078</v>
       </c>
       <c r="F40" t="n">
-        <v>1536</v>
+        <v>799</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>BN-GC-7-nn</t>
+          <t>BN-IDC-2-1-nn</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1553,25 +1553,25 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-nn/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-1-nn/002.jpg</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-nn\002_image_BN-GC-7-nn.jpg</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-1-nn\2_image_BN-IDC-2-1-nn.png</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>2752</v>
+        <v>1161</v>
       </c>
       <c r="F41" t="n">
-        <v>1536</v>
+        <v>741</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>BN-GC-7-o</t>
+          <t>BN-OP-23-1-k</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1581,25 +1581,25 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-o/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-1-k/002.jpg</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-o\002_image_BN-GC-7-o.jpg</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-1-k\2_image_BN-OP-23-1-k.png</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>2752</v>
+        <v>1447</v>
       </c>
       <c r="F42" t="n">
-        <v>1536</v>
+        <v>672</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>BN-GC-7-red</t>
+          <t>BN-OP-23-1-navy-blue</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1609,25 +1609,25 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-red/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-1-navy-blue/002.jpg</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-red\002_image_BN-GC-7-red.jpg</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-1-navy-blue\2_image_BN-OP-23-1-navy-blue.png</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>2752</v>
+        <v>1274</v>
       </c>
       <c r="F43" t="n">
-        <v>1536</v>
+        <v>942</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>BN-GC-7-tiffany</t>
+          <t>BN-OP-23-beige</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1637,25 +1637,25 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-tiffany/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-beige/002.jpg</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-tiffany\002_image_BN-GC-7-tiffany.jpg</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-beige\2_image_BN-OP-23-beige.png</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>2752</v>
+        <v>1274</v>
       </c>
       <c r="F44" t="n">
-        <v>1536</v>
+        <v>942</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>BN-GC-7-vin</t>
+          <t>BN-OP-23-choko</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1665,25 +1665,25 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-vin/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-choko/002.jpg</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-vin\002_image_BN-GC-7-vin.jpg</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-choko\2_image_BN-OP-23-choko.png</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>2752</v>
+        <v>1069</v>
       </c>
       <c r="F45" t="n">
-        <v>1536</v>
+        <v>703</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>BN-GC-7-vin-kr</t>
+          <t>BN-OP-23-g</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1693,25 +1693,25 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-vin-kr/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-g/002.jpg</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-vin-kr\002_image_BN-GC-7-vin-kr.jpg</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-g\2_image_BN-OP-23-g.png</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>2752</v>
+        <v>1319</v>
       </c>
       <c r="F46" t="n">
-        <v>1536</v>
+        <v>732</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>BN-GC-8-g-kr</t>
+          <t>BN-OP-23-malachite</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1721,25 +1721,25 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-8-g-kr/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-malachite/002.jpg</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-8-g-kr\002_image_BN-GC-8-g-kr.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-malachite\2_image_BN-OP-23-malachite.png</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>1482</v>
+        <v>1111</v>
       </c>
       <c r="F47" t="n">
-        <v>1062</v>
+        <v>717</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>BN-GC-8-k-kr</t>
+          <t>BN-OP-25-1-g</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1749,25 +1749,25 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-8-k-kr/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-g/002.jpg</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-8-k-kr\002_image_BN-GC-8-k-kr.jpg</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-g\2_image_BN-OP-25-1-g.png</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>2752</v>
+        <v>1182</v>
       </c>
       <c r="F48" t="n">
-        <v>1536</v>
+        <v>836</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>BN-GC-8-o</t>
+          <t>BN-OP-25-1-k</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1777,193 +1777,193 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-8-o/002.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-k/002.jpg</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-8-o\002_image_BN-GC-8-o.jpg</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-k\2_image_BN-OP-25-1-k.png</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>2752</v>
+        <v>1192</v>
       </c>
       <c r="F49" t="n">
-        <v>1536</v>
+        <v>1088</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>BN-GC-7-g-kr</t>
+          <t>BN-OP-25-1-light-beige</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>003.jpg</t>
+          <t>002.jpg</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-g-kr/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-light-beige/002.jpg</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-g-kr\3_image_BN-GC-7-g-kr.jpg</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-light-beige\2_image_BN-OP-25-1-light-beige.png</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>2752</v>
+        <v>811</v>
       </c>
       <c r="F50" t="n">
-        <v>1536</v>
+        <v>949</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>BN-GC-7-k</t>
+          <t>BN-OP-25-1-malachite</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>003.jpg</t>
+          <t>002.jpg</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-k/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-malachite/002.jpg</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-k\003_image_BN-GC-7-k.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-malachite\2_image_BN-OP-25-1-malachite.png</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>1483</v>
+        <v>1240</v>
       </c>
       <c r="F51" t="n">
-        <v>1061</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>BN-GC-7-k-kr</t>
+          <t>BN-OP-25-1-navy-blue</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>003.jpg</t>
+          <t>002.jpg</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-k-kr/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-navy-blue/002.jpg</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-k-kr\003_image_BN-GC-7-k-kr.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-navy-blue\2_image_BN-OP-25-1-navy-blue.png</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>1482</v>
+        <v>1284</v>
       </c>
       <c r="F52" t="n">
-        <v>1062</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>BN-GC-7-malachite</t>
+          <t>BN-OP-25-malachite</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>003.jpg</t>
+          <t>002.jpg</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-malachite/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-malachite/002.jpg</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-malachite\3_image_BN-GC-7-malachite.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-malachite\2_image_BN-OP-25-malachite.png</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>1482</v>
+        <v>1127</v>
       </c>
       <c r="F53" t="n">
-        <v>1061</v>
+        <v>869</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>BN-GC-7-navy-blue</t>
+          <t>BN-OP-25-navy-blue</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>003.jpg</t>
+          <t>002.jpg</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-navy-blue/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-navy-blue/002.jpg</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-navy-blue\3_image_BN-GC-7-navy-blue.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-navy-blue\2_image_BN-OP-25-navy-blue.png</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>1482</v>
+        <v>1128</v>
       </c>
       <c r="F54" t="n">
-        <v>1061</v>
+        <v>848</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>BN-GC-7-nn</t>
+          <t>BN-OP-26-light</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>003.jpg</t>
+          <t>002.jpg</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-nn/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-26-light/002.jpg</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-nn\3_image_BN-GC-7-nn.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-26-light\2_image_BN-OP-26-light.png</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>1482</v>
+        <v>904</v>
       </c>
       <c r="F55" t="n">
-        <v>1061</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>BN-GC-7-o</t>
+          <t>BN-IDC-1-g</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1973,25 +1973,25 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-o/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-1-g/003.jpg</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-o\003_image_BN-GC-7-o.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-1-g\3_image_BN-IDC-1-g.png</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>1482</v>
+        <v>530</v>
       </c>
       <c r="F56" t="n">
-        <v>1061</v>
+        <v>1743</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>BN-GC-7-red</t>
+          <t>BN-IDC-2-1-g-kr</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2001,25 +2001,25 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-red/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-1-g-kr/003.jpg</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-red\3_image_BN-GC-7-red.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-1-g-kr\3_image_BN-IDC-2-1-g-kr.png</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>1482</v>
+        <v>1118</v>
       </c>
       <c r="F57" t="n">
-        <v>1061</v>
+        <v>776</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>BN-GC-7-tiffany</t>
+          <t>BN-IDC-2-1-k-kr</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2029,25 +2029,25 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-tiffany/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-1-k-kr/003.jpg</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-tiffany\003_image_BN-GC-7-tiffany.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-1-k-kr\3_image_BN-IDC-2-1-k-kr.png</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>1482</v>
+        <v>1092</v>
       </c>
       <c r="F58" t="n">
-        <v>1061</v>
+        <v>813</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>BN-GC-7-vin</t>
+          <t>BN-IDC-2-1-malachite</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2057,25 +2057,25 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-vin/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-1-malachite/003.jpg</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-vin\003_image_BN-GC-7-vin.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-1-malachite\3_image_BN-IDC-2-1-malachite.png</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>1483</v>
+        <v>1121</v>
       </c>
       <c r="F59" t="n">
-        <v>1061</v>
+        <v>769</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>BN-GC-7-vin-kr</t>
+          <t>BN-IDC-2-1-navy-blue</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2085,25 +2085,25 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-vin-kr/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-1-navy-blue/003.jpg</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-vin-kr\3_image_BN-GC-7-vin-kr.jpg</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-1-navy-blue\3_image_BN-IDC-2-1-navy-blue.png</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>2752</v>
+        <v>1107</v>
       </c>
       <c r="F60" t="n">
-        <v>1536</v>
+        <v>785</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>BN-GC-8-k-kr</t>
+          <t>BN-IDC-2-1-o</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2113,25 +2113,25 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-8-k-kr/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-1-o/003.jpg</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-8-k-kr\003_image_BN-GC-8-k-kr.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-1-o\3_image_BN-IDC-2-1-o.png</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>1483</v>
+        <v>1090</v>
       </c>
       <c r="F61" t="n">
-        <v>1061</v>
+        <v>738</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>BN-GC-8-o</t>
+          <t>BN-IDC-2-1-red</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2141,439 +2141,2679 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-8-o/003.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-1-red/003.jpg</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-8-o\3_image_BN-GC-8-o.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-1-red\3_image_BN-IDC-2-1-red.png</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>1483</v>
+        <v>1143</v>
       </c>
       <c r="F62" t="n">
-        <v>1061</v>
+        <v>775</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>BN-GC-19-g-kr</t>
+          <t>BN-IDC-2-2-beige-kr</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>004.jpg</t>
+          <t>003.jpg</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-19-g-kr/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-2-beige-kr/003.jpg</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-19-g-kr\004_image_BN-GC-19-g-kr.jpg</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-2-beige-kr\3_image_BN-IDC-2-2-beige-kr.png</t>
         </is>
       </c>
       <c r="E63" t="n">
-        <v>2752</v>
+        <v>979</v>
       </c>
       <c r="F63" t="n">
-        <v>1536</v>
+        <v>737</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>BN-GC-19-iz</t>
+          <t>BN-IDC-2-2-choko</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>004.jpg</t>
+          <t>003.jpg</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-19-iz/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-2-choko/003.jpg</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-19-iz\004_image_BN-GC-19-iz.jpg</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-2-choko\3_image_BN-IDC-2-2-choko.png</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>2752</v>
+        <v>1005</v>
       </c>
       <c r="F64" t="n">
-        <v>1536</v>
+        <v>751</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>BN-GC-19-k-kr</t>
+          <t>BN-IDC-2-2-g-kr</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>004.jpg</t>
+          <t>003.jpg</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-19-k-kr/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-2-g-kr/003.jpg</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-19-k-kr\004_image_BN-GC-19-k-kr.jpg</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-2-g-kr\3_image_BN-IDC-2-2-g-kr.png</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>2752</v>
+        <v>1000</v>
       </c>
       <c r="F65" t="n">
-        <v>1536</v>
+        <v>735</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>BN-GC-19-o</t>
+          <t>BN-IDC-2-2-iz</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>004.jpg</t>
+          <t>003.jpg</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-19-o/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-2-iz/003.jpg</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-19-o\004_image_BN-GC-19-o.jpg</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-2-iz\3_image_BN-IDC-2-2-iz.png</t>
         </is>
       </c>
       <c r="E66" t="n">
-        <v>2752</v>
+        <v>1075</v>
       </c>
       <c r="F66" t="n">
-        <v>1536</v>
+        <v>759</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>BN-GC-19-vin-kr</t>
+          <t>BN-IDC-2-2-k-kr</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>004.jpg</t>
+          <t>003.jpg</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-19-vin-kr/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-2-k-kr/003.jpg</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-19-vin-kr\004_image_BN-GC-19-vin-kr.jpg</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-2-k-kr\3_image_BN-IDC-2-2-k-kr.png</t>
         </is>
       </c>
       <c r="E67" t="n">
-        <v>2752</v>
+        <v>1015</v>
       </c>
       <c r="F67" t="n">
-        <v>1536</v>
+        <v>733</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>BN-GC-28-choko</t>
+          <t>BN-IDC-2-2-malachite</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>004.jpg</t>
+          <t>003.jpg</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-28-choko/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-2-malachite/003.jpg</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-28-choko\004_image_BN-GC-28-choko.jpg</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-2-malachite\3_image_BN-IDC-2-2-malachite.png</t>
         </is>
       </c>
       <c r="E68" t="n">
-        <v>2752</v>
+        <v>1113</v>
       </c>
       <c r="F68" t="n">
-        <v>1536</v>
+        <v>748</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>BN-GC-28-g</t>
+          <t>BN-IDC-2-2-nn</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>004.jpg</t>
+          <t>003.jpg</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-28-g/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-2-nn/003.jpg</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-28-g\004_image_BN-GC-28-g.jpg</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-2-nn\3_image_BN-IDC-2-2-nn.png</t>
         </is>
       </c>
       <c r="E69" t="n">
-        <v>2752</v>
+        <v>1003</v>
       </c>
       <c r="F69" t="n">
-        <v>1536</v>
+        <v>754</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>BN-GC-28-k</t>
+          <t>BN-IDC-2-2-o</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>004.jpg</t>
+          <t>003.jpg</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-28-k/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-2-o/003.jpg</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-28-k\004_image_BN-GC-28-k.jpg</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-2-o\3_image_BN-IDC-2-2-o.png</t>
         </is>
       </c>
       <c r="E70" t="n">
-        <v>2752</v>
+        <v>902</v>
       </c>
       <c r="F70" t="n">
-        <v>1536</v>
+        <v>751</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>BN-GC-28-malachite</t>
+          <t>BN-OP-23-1-malachite</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>004.jpg</t>
+          <t>003.jpg</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-28-malachite/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-1-malachite/003.jpg</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-28-malachite\004_image_BN-GC-28-malachite.jpg</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-1-malachite\3_image_BN-OP-23-1-malachite.png</t>
         </is>
       </c>
       <c r="E71" t="n">
-        <v>2752</v>
+        <v>1365</v>
       </c>
       <c r="F71" t="n">
-        <v>1536</v>
+        <v>649</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>BN-GC-7-iz</t>
+          <t>BN-OP-23-1-navy-blue</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>004.jpg</t>
+          <t>003.jpg</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-iz/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-1-navy-blue/003.jpg</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-iz\004_image_BN-GC-7-iz.jpg</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-1-navy-blue\3_image_BN-OP-23-1-navy-blue.png</t>
         </is>
       </c>
       <c r="E72" t="n">
-        <v>2752</v>
+        <v>1103</v>
       </c>
       <c r="F72" t="n">
-        <v>1536</v>
+        <v>685</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>BN-GC-7-k-kr</t>
+          <t>BN-OP-23-beige</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>004.jpg</t>
+          <t>003.jpg</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-k-kr/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-beige/003.jpg</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-k-kr\4_image_BN-GC-7-k-kr.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-beige\3_image_BN-OP-23-beige.png</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>1483</v>
+        <v>1364</v>
       </c>
       <c r="F73" t="n">
-        <v>1061</v>
+        <v>735</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>BN-GC-7-malachite</t>
+          <t>BN-OP-23-choko</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>004.jpg</t>
+          <t>003.jpg</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-malachite/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-choko/003.jpg</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-malachite\004_image_BN-GC-7-malachite.png</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-choko\3_image_BN-OP-23-choko.png</t>
         </is>
       </c>
       <c r="E74" t="n">
-        <v>1482</v>
+        <v>1372</v>
       </c>
       <c r="F74" t="n">
-        <v>1061</v>
+        <v>753</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>BN-GC-8-g-kr</t>
+          <t>BN-OP-23-g</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>004.jpg</t>
+          <t>003.jpg</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-8-g-kr/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-g/003.jpg</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-8-g-kr\004_image_BN-GC-8-g-kr.jpg</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-g\3_image_BN-OP-23-g.png</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>2752</v>
+        <v>1034</v>
       </c>
       <c r="F75" t="n">
-        <v>1536</v>
+        <v>695</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>BN-GC-7-k</t>
+          <t>BN-OP-23-k</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>005.jpg</t>
+          <t>003.jpg</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-k/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-k/003.jpg</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-k\005_image_BN-GC-7-k.jpg</t>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-k\3_image_BN-OP-23-k.png</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>2752</v>
+        <v>942</v>
       </c>
       <c r="F76" t="n">
-        <v>1536</v>
+        <v>783</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>BN-GC-7-vin-kr</t>
+          <t>BN-OP-23-malachite</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
+          <t>003.jpg</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-malachite/003.jpg</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-malachite\3_image_BN-OP-23-malachite.png</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>1164</v>
+      </c>
+      <c r="F77" t="n">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>BN-OP-23-navy-blue</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>003.jpg</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-navy-blue/003.jpg</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-navy-blue\3_image_BN-OP-23-navy-blue.png</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>1096</v>
+      </c>
+      <c r="F78" t="n">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>BN-OP-25-1-choko</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>003.jpg</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-choko/003.jpg</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-choko\3_image_BN-OP-25-1-choko.png</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>1164</v>
+      </c>
+      <c r="F79" t="n">
+        <v>1107</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>BN-OP-25-1-g</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>003.jpg</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-g/003.jpg</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-g\3_image_BN-OP-25-1-g.png</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>1175</v>
+      </c>
+      <c r="F80" t="n">
+        <v>871</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>BN-OP-25-1-k</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>003.jpg</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-k/003.jpg</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-k\3_image_BN-OP-25-1-k.png</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>1182</v>
+      </c>
+      <c r="F81" t="n">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>BN-OP-25-1-light-beige</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>003.jpg</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-light-beige/003.jpg</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-light-beige\3_image_BN-OP-25-1-light-beige.png</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>1294</v>
+      </c>
+      <c r="F82" t="n">
+        <v>873</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>BN-OP-25-1-malachite</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>003.jpg</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-malachite/003.jpg</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-malachite\3_image_BN-OP-25-1-malachite.png</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>799</v>
+      </c>
+      <c r="F83" t="n">
+        <v>906</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>BN-OP-25-1-navy-blue</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>003.jpg</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-navy-blue/003.jpg</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-navy-blue\3_image_BN-OP-25-1-navy-blue.png</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>1264</v>
+      </c>
+      <c r="F84" t="n">
+        <v>837</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>BN-OP-25-g-kr</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>003.jpg</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-g-kr/003.jpg</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-g-kr\3_image_BN-OP-25-g-kr.png</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>1148</v>
+      </c>
+      <c r="F85" t="n">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>BN-OP-25-malachite</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>003.jpg</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-malachite/003.jpg</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-malachite\3_image_BN-OP-25-malachite.png</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>1144</v>
+      </c>
+      <c r="F86" t="n">
+        <v>843</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>BN-OP-26-k</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>003.jpg</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-26-k/003.jpg</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-26-k\003_image_BN-OP-26-k.png</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>1167</v>
+      </c>
+      <c r="F87" t="n">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>BN-IDC-1-g</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-1-g/004.jpg</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-1-g\4_image_BN-IDC-1-g.png</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>737</v>
+      </c>
+      <c r="F88" t="n">
+        <v>1476</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>BN-IDC-2-1-beige-kr</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-1-beige-kr/004.jpg</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-1-beige-kr\004_image_BN-IDC-2-1-beige-kr.png</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>1389</v>
+      </c>
+      <c r="F89" t="n">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>BN-IDC-2-1-g-kr</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-1-g-kr/004.jpg</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-1-g-kr\004_image_BN-IDC-2-1-g-kr.png</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>1416</v>
+      </c>
+      <c r="F90" t="n">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>BN-IDC-2-1-k-kr</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-1-k-kr/004.jpg</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-1-k-kr\004_image_BN-IDC-2-1-k-kr.png</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>1443</v>
+      </c>
+      <c r="F91" t="n">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>BN-IDC-2-1-malachite</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-1-malachite/004.jpg</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-1-malachite\004_image_BN-IDC-2-1-malachite.png</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>1130</v>
+      </c>
+      <c r="F92" t="n">
+        <v>823</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>BN-IDC-2-1-navy-blue</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-1-navy-blue/004.jpg</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-1-navy-blue\004_image_BN-IDC-2-1-navy-blue.png</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>1461</v>
+      </c>
+      <c r="F93" t="n">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>BN-IDC-2-1-nn</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-1-nn/004.jpg</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-1-nn\004_image_BN-IDC-2-1-nn.png</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>1435</v>
+      </c>
+      <c r="F94" t="n">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>BN-IDC-2-1-o</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-1-o/004.jpg</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-1-o\004_image_BN-IDC-2-1-o.png</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>1456</v>
+      </c>
+      <c r="F95" t="n">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>BN-IDC-2-1-red</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-1-red/004.jpg</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-1-red\004_image_BN-IDC-2-1-red.png</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>1461</v>
+      </c>
+      <c r="F96" t="n">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>BN-IDC-2-2-beige-kr</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-2-beige-kr/004.jpg</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-2-beige-kr\004_image_BN-IDC-2-2-beige-kr.png</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>1442</v>
+      </c>
+      <c r="F97" t="n">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>BN-IDC-2-2-choko</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-2-choko/004.jpg</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-2-choko\004_image_BN-IDC-2-2-choko.png</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>1432</v>
+      </c>
+      <c r="F98" t="n">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>BN-IDC-2-2-g-kr</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-2-g-kr/004.jpg</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-2-g-kr\004_image_BN-IDC-2-2-g-kr.png</t>
+        </is>
+      </c>
+      <c r="E99" t="n">
+        <v>1446</v>
+      </c>
+      <c r="F99" t="n">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>BN-IDC-2-2-iz</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-2-iz/004.jpg</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-2-iz\004_image_BN-IDC-2-2-iz.png</t>
+        </is>
+      </c>
+      <c r="E100" t="n">
+        <v>1450</v>
+      </c>
+      <c r="F100" t="n">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>BN-IDC-2-2-k-kr</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-2-k-kr/004.jpg</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-2-k-kr\004_image_BN-IDC-2-2-k-kr.png</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>1467</v>
+      </c>
+      <c r="F101" t="n">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>BN-IDC-2-2-malachite</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-2-malachite/004.jpg</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-2-malachite\004_image_BN-IDC-2-2-malachite.png</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>1458</v>
+      </c>
+      <c r="F102" t="n">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>BN-IDC-2-2-nn</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-2-nn/004.jpg</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-2-nn\004_image_BN-IDC-2-2-nn.png</t>
+        </is>
+      </c>
+      <c r="E103" t="n">
+        <v>1469</v>
+      </c>
+      <c r="F103" t="n">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>BN-IDC-2-2-o</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-2-o/004.jpg</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-2-o\4_image_BN-IDC-2-2-o.png</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>1036</v>
+      </c>
+      <c r="F104" t="n">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>BN-OP-23-1-k</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-1-k/004.jpg</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-1-k\4_image_BN-OP-23-1-k.png</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>1088</v>
+      </c>
+      <c r="F105" t="n">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>BN-OP-23-1-malachite</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-1-malachite/004.jpg</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-1-malachite\4_image_BN-OP-23-1-malachite.png</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>1343</v>
+      </c>
+      <c r="F106" t="n">
+        <v>975</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>BN-OP-23-1-navy-blue</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-1-navy-blue/004.jpg</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-1-navy-blue\4_image_BN-OP-23-1-navy-blue.png</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>1370</v>
+      </c>
+      <c r="F107" t="n">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>BN-OP-23-beige</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-beige/004.jpg</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-beige\4_image_BN-OP-23-beige.png</t>
+        </is>
+      </c>
+      <c r="E108" t="n">
+        <v>1366</v>
+      </c>
+      <c r="F108" t="n">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>BN-OP-23-choko</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-choko/004.jpg</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-choko\4_image_BN-OP-23-choko.png</t>
+        </is>
+      </c>
+      <c r="E109" t="n">
+        <v>1400</v>
+      </c>
+      <c r="F109" t="n">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>BN-OP-23-g</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-g/004.jpg</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-g\4_image_BN-OP-23-g.png</t>
+        </is>
+      </c>
+      <c r="E110" t="n">
+        <v>1320</v>
+      </c>
+      <c r="F110" t="n">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>BN-OP-23-k</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-k/004.jpg</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-k\4_image_BN-OP-23-k.png</t>
+        </is>
+      </c>
+      <c r="E111" t="n">
+        <v>1192</v>
+      </c>
+      <c r="F111" t="n">
+        <v>894</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>BN-OP-23-malachite</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-malachite/004.jpg</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-malachite\4_image_BN-OP-23-malachite.png</t>
+        </is>
+      </c>
+      <c r="E112" t="n">
+        <v>1188</v>
+      </c>
+      <c r="F112" t="n">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>BN-OP-23-navy-blue</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-navy-blue/004.jpg</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-navy-blue\4_image_BN-OP-23-navy-blue.png</t>
+        </is>
+      </c>
+      <c r="E113" t="n">
+        <v>1220</v>
+      </c>
+      <c r="F113" t="n">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>BN-OP-25-1-choko</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-choko/004.jpg</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-choko\4_image_BN-OP-25-1-choko.png</t>
+        </is>
+      </c>
+      <c r="E114" t="n">
+        <v>1135</v>
+      </c>
+      <c r="F114" t="n">
+        <v>854</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>BN-OP-25-1-g</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-g/004.jpg</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-g\4_image_BN-OP-25-1-g.png</t>
+        </is>
+      </c>
+      <c r="E115" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F115" t="n">
+        <v>848</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>BN-OP-25-1-k</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-k/004.jpg</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-k\4_image_BN-OP-25-1-k.png</t>
+        </is>
+      </c>
+      <c r="E116" t="n">
+        <v>827</v>
+      </c>
+      <c r="F116" t="n">
+        <v>962</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>BN-OP-25-1-light-beige</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-light-beige/004.jpg</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-light-beige\4_image_BN-OP-25-1-light-beige.png</t>
+        </is>
+      </c>
+      <c r="E117" t="n">
+        <v>1170</v>
+      </c>
+      <c r="F117" t="n">
+        <v>887</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>BN-OP-25-1-malachite</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-malachite/004.jpg</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-malachite\4_image_BN-OP-25-1-malachite.png</t>
+        </is>
+      </c>
+      <c r="E118" t="n">
+        <v>1275</v>
+      </c>
+      <c r="F118" t="n">
+        <v>921</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>BN-OP-25-1-navy-blue</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-navy-blue/004.jpg</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-navy-blue\4_image_BN-OP-25-1-navy-blue.png</t>
+        </is>
+      </c>
+      <c r="E119" t="n">
+        <v>1306</v>
+      </c>
+      <c r="F119" t="n">
+        <v>848</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>BN-OP-25-g-kr</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-g-kr/004.jpg</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-g-kr\4_image_BN-OP-25-g-kr.png</t>
+        </is>
+      </c>
+      <c r="E120" t="n">
+        <v>1131</v>
+      </c>
+      <c r="F120" t="n">
+        <v>861</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>BN-OP-25-malachite</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-malachite/004.jpg</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-malachite\4_image_BN-OP-25-malachite.png</t>
+        </is>
+      </c>
+      <c r="E121" t="n">
+        <v>812</v>
+      </c>
+      <c r="F121" t="n">
+        <v>946</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>BN-OP-25-navy-blue</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-navy-blue/004.jpg</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-navy-blue\4_image_BN-OP-25-navy-blue.png</t>
+        </is>
+      </c>
+      <c r="E122" t="n">
+        <v>757</v>
+      </c>
+      <c r="F122" t="n">
+        <v>911</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>BN-OP-26-light</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>004.jpg</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-26-light/004.jpg</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-26-light\4_image_BN-OP-26-light.png</t>
+        </is>
+      </c>
+      <c r="E123" t="n">
+        <v>840</v>
+      </c>
+      <c r="F123" t="n">
+        <v>1122</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>BN-IDC-1-g</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
           <t>005.jpg</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-vin-kr/005.jpg</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>C:/Users/Asus/Desktop/чохли обєднання/додавання фото/2 перейменовані фото/result_2026-10-25_18-22-51\BN-GC-7-vin-kr\005_image_BN-GC-7-vin-kr.jpg</t>
-        </is>
-      </c>
-      <c r="E77" t="n">
-        <v>2390</v>
-      </c>
-      <c r="F77" t="n">
-        <v>1760</v>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-1-g/005.jpg</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-1-g\5_image_BN-IDC-1-g.png</t>
+        </is>
+      </c>
+      <c r="E124" t="n">
+        <v>560</v>
+      </c>
+      <c r="F124" t="n">
+        <v>1326</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>BN-IDC-2-2-o</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>005.jpg</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-2-2-o/005.jpg</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-2-2-o\005_image_BN-IDC-2-2-o.png</t>
+        </is>
+      </c>
+      <c r="E125" t="n">
+        <v>1435</v>
+      </c>
+      <c r="F125" t="n">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>BN-OP-23-1-k</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>005.jpg</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-1-k/005.jpg</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-1-k\005_image_BN-OP-23-1-k.png</t>
+        </is>
+      </c>
+      <c r="E126" t="n">
+        <v>1428</v>
+      </c>
+      <c r="F126" t="n">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>BN-OP-23-1-malachite</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>005.jpg</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-1-malachite/005.jpg</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-1-malachite\5_image_BN-OP-23-1-malachite.png</t>
+        </is>
+      </c>
+      <c r="E127" t="n">
+        <v>1402</v>
+      </c>
+      <c r="F127" t="n">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>BN-OP-23-1-navy-blue</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>005.jpg</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-1-navy-blue/005.jpg</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-1-navy-blue\5_image_BN-OP-23-1-navy-blue.png</t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>1372</v>
+      </c>
+      <c r="F128" t="n">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>BN-OP-23-beige</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>005.jpg</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-beige/005.jpg</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-beige\5_image_BN-OP-23-beige.png</t>
+        </is>
+      </c>
+      <c r="E129" t="n">
+        <v>995</v>
+      </c>
+      <c r="F129" t="n">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>BN-OP-23-choko</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>005.jpg</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-choko/005.jpg</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-choko\5_image_BN-OP-23-choko.png</t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>1357</v>
+      </c>
+      <c r="F130" t="n">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>BN-OP-23-g</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>005.jpg</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-g/005.jpg</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-g\5_image_BN-OP-23-g.png</t>
+        </is>
+      </c>
+      <c r="E131" t="n">
+        <v>1351</v>
+      </c>
+      <c r="F131" t="n">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>BN-OP-23-k</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>005.jpg</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-k/005.jpg</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-k\5_image_BN-OP-23-k.png</t>
+        </is>
+      </c>
+      <c r="E132" t="n">
+        <v>1140</v>
+      </c>
+      <c r="F132" t="n">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>BN-OP-23-malachite</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>005.jpg</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-malachite/005.jpg</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-malachite\5_image_BN-OP-23-malachite.png</t>
+        </is>
+      </c>
+      <c r="E133" t="n">
+        <v>1193</v>
+      </c>
+      <c r="F133" t="n">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>BN-OP-23-navy-blue</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>005.jpg</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-navy-blue/005.jpg</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-navy-blue\5_image_BN-OP-23-navy-blue.png</t>
+        </is>
+      </c>
+      <c r="E134" t="n">
+        <v>1213</v>
+      </c>
+      <c r="F134" t="n">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>BN-OP-25-1-choko</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>005.jpg</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-choko/005.jpg</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-choko\5_image_BN-OP-25-1-choko.png</t>
+        </is>
+      </c>
+      <c r="E135" t="n">
+        <v>1119</v>
+      </c>
+      <c r="F135" t="n">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>BN-OP-25-1-g</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>005.jpg</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-g/005.jpg</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-g\5_image_BN-OP-25-1-g.png</t>
+        </is>
+      </c>
+      <c r="E136" t="n">
+        <v>1089</v>
+      </c>
+      <c r="F136" t="n">
+        <v>1060</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>BN-OP-25-1-k</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>005.jpg</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-k/005.jpg</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-k\5_image_BN-OP-25-1-k.png</t>
+        </is>
+      </c>
+      <c r="E137" t="n">
+        <v>1287</v>
+      </c>
+      <c r="F137" t="n">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>BN-OP-25-1-malachite</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>005.jpg</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-malachite/005.jpg</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-malachite\5_image_BN-OP-25-1-malachite.png</t>
+        </is>
+      </c>
+      <c r="E138" t="n">
+        <v>1295</v>
+      </c>
+      <c r="F138" t="n">
+        <v>884</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>BN-OP-25-1-navy-blue</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>005.jpg</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-navy-blue/005.jpg</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-navy-blue\5_image_BN-OP-25-1-navy-blue.png</t>
+        </is>
+      </c>
+      <c r="E139" t="n">
+        <v>1280</v>
+      </c>
+      <c r="F139" t="n">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>BN-OP-25-g-kr</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>005.jpg</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-g-kr/005.jpg</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-g-kr\5_image_BN-OP-25-g-kr.png</t>
+        </is>
+      </c>
+      <c r="E140" t="n">
+        <v>842</v>
+      </c>
+      <c r="F140" t="n">
+        <v>963</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>BN-OP-25-navy-blue</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>005.jpg</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-navy-blue/005.jpg</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-navy-blue\5_image_BN-OP-25-navy-blue.png</t>
+        </is>
+      </c>
+      <c r="E141" t="n">
+        <v>1125</v>
+      </c>
+      <c r="F141" t="n">
+        <v>908</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>BN-OP-26-light</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>005.jpg</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-26-light/005.jpg</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-26-light\005_image_BN-OP-26-light.png</t>
+        </is>
+      </c>
+      <c r="E142" t="n">
+        <v>1167</v>
+      </c>
+      <c r="F142" t="n">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>BN-OP-23-1-malachite</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>006.jpg</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-1-malachite/006.jpg</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-1-malachite\006_image_BN-OP-23-1-malachite.png</t>
+        </is>
+      </c>
+      <c r="E143" t="n">
+        <v>1005</v>
+      </c>
+      <c r="F143" t="n">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>BN-OP-23-beige</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>006.jpg</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-beige/006.jpg</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-beige\6_image_BN-OP-23-beige.png</t>
+        </is>
+      </c>
+      <c r="E144" t="n">
+        <v>1371</v>
+      </c>
+      <c r="F144" t="n">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>BN-OP-23-k</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>006.jpg</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-k/006.jpg</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-k\6_image_BN-OP-23-k.png</t>
+        </is>
+      </c>
+      <c r="E145" t="n">
+        <v>1122</v>
+      </c>
+      <c r="F145" t="n">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>BN-OP-23-navy-blue</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>006.jpg</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-navy-blue/006.jpg</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-navy-blue\006_image_BN-OP-23-navy-blue.png</t>
+        </is>
+      </c>
+      <c r="E146" t="n">
+        <v>1196</v>
+      </c>
+      <c r="F146" t="n">
+        <v>721</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>BN-OP-25-1-choko</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>006.jpg</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-choko/006.jpg</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-choko\6_image_BN-OP-25-1-choko.png</t>
+        </is>
+      </c>
+      <c r="E147" t="n">
+        <v>1167</v>
+      </c>
+      <c r="F147" t="n">
+        <v>819</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>BN-OP-25-1-malachite</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>006.jpg</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-malachite/006.jpg</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-malachite\6_image_BN-OP-25-1-malachite.png</t>
+        </is>
+      </c>
+      <c r="E148" t="n">
+        <v>1350</v>
+      </c>
+      <c r="F148" t="n">
+        <v>880</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>BN-OP-25-g-kr</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>006.jpg</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-g-kr/006.jpg</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-g-kr\006_image_BN-OP-25-g-kr.png</t>
+        </is>
+      </c>
+      <c r="E149" t="n">
+        <v>1150</v>
+      </c>
+      <c r="F149" t="n">
+        <v>852</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>BN-OP-25-navy-blue</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>006.jpg</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-navy-blue/006.jpg</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-navy-blue\006_image_BN-OP-25-navy-blue.png</t>
+        </is>
+      </c>
+      <c r="E150" t="n">
+        <v>1123</v>
+      </c>
+      <c r="F150" t="n">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>BN-IDC-1-g</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>007.jpg</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-IDC-1-g/007.jpg</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-IDC-1-g\007_image_BN-IDC-1-g.png</t>
+        </is>
+      </c>
+      <c r="E151" t="n">
+        <v>530</v>
+      </c>
+      <c r="F151" t="n">
+        <v>1801</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>BN-OP-23-k</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>007.jpg</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-k/007.jpg</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-k\7_image_BN-OP-23-k.png</t>
+        </is>
+      </c>
+      <c r="E152" t="n">
+        <v>1144</v>
+      </c>
+      <c r="F152" t="n">
+        <v>696</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>BN-OP-25-1-choko</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>007.jpg</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-25-1-choko/007.jpg</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-25-1-choko\007_image_BN-OP-25-1-choko.png</t>
+        </is>
+      </c>
+      <c r="E153" t="n">
+        <v>921</v>
+      </c>
+      <c r="F153" t="n">
+        <v>1031</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>BN-OP-23-k</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>008.jpg</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-k/008.jpg</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-k\8_image_BN-OP-23-k.png</t>
+        </is>
+      </c>
+      <c r="E154" t="n">
+        <v>1105</v>
+      </c>
+      <c r="F154" t="n">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>BN-OP-23-k</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>009.jpg</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-k/009.jpg</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-k\9_image_BN-OP-23-k.png</t>
+        </is>
+      </c>
+      <c r="E155" t="n">
+        <v>1092</v>
+      </c>
+      <c r="F155" t="n">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>BN-OP-23-k</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>010.jpg</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-k/010.jpg</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-k\10_image_BN-OP-23-k.png</t>
+        </is>
+      </c>
+      <c r="E156" t="n">
+        <v>1016</v>
+      </c>
+      <c r="F156" t="n">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>BN-OP-23-k</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>011.jpg</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-OP-23-k/011.jpg</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>D:/Спільна папка/2 Редагування/1 обкладинки для Каста/фото/залиті фото/обрізані\BN-OP-23-k\011_image_BN-OP-23-k.png</t>
+        </is>
+      </c>
+      <c r="E157" t="n">
+        <v>1124</v>
+      </c>
+      <c r="F157" t="n">
+        <v>773</v>
       </c>
     </row>
   </sheetData>

</xml_diff>